<commit_message>
merged-cells: partially working range accumulations
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Excell_T1_small.xlsx
+++ b/Ref_Files/Test_Excell_T1_small.xlsx
@@ -1048,7 +1048,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="25" t="n">
-        <v>100</v>
+        <v>555</v>
       </c>
       <c r="E12" s="25"/>
       <c r="F12" s="25"/>
@@ -1090,7 +1090,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>100</v>
+        <v>11</v>
       </c>
       <c r="E15" s="25"/>
       <c r="F15" s="25"/>
@@ -1156,7 +1156,7 @@
         <v>18</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>100</v>
+        <v>11</v>
       </c>
       <c r="E19" s="25"/>
       <c r="F19" s="25"/>
@@ -1222,7 +1222,7 @@
         <v>18</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>100</v>
+        <v>11</v>
       </c>
       <c r="E23" s="25"/>
       <c r="F23" s="25"/>

</xml_diff>